<commit_message>
Finished practise part of project
</commit_message>
<xml_diff>
--- a/Other/testexample.xlsx
+++ b/Other/testexample.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29825"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29905"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{80757F05-05C6-4A77-B35C-E98ACD4ABB44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{24E3CE0B-5717-429C-AE00-209986D55C5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,26 +30,64 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={1661D921-632C-430C-921D-9910BCE3059E}</author>
+    <author>tc={955AFFB0-AFFE-458F-8DA4-B07AF093579C}</author>
+    <author>tc={BFCD12D3-2FD0-414A-BD87-6586BD3166F9}</author>
+  </authors>
+  <commentList>
+    <comment ref="A2" authorId="0" shapeId="0" xr:uid="{1661D921-632C-430C-921D-9910BCE3059E}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    писать вопрос здесь, а справа ответ на него
+(так можно писать вниз до бесконечности)</t>
+      </text>
+    </comment>
+    <comment ref="C2" authorId="1" shapeId="0" xr:uid="{955AFFB0-AFFE-458F-8DA4-B07AF093579C}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    писать название здесь</t>
+      </text>
+    </comment>
+    <comment ref="D2" authorId="2" shapeId="0" xr:uid="{BFCD12D3-2FD0-414A-BD87-6586BD3166F9}">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    писать тему здесь
+</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+  <si>
+    <t>Question</t>
+  </si>
+  <si>
+    <t>Answer</t>
+  </si>
   <si>
     <t>TestName</t>
   </si>
   <si>
     <t>TestTheme</t>
   </si>
-  <si>
-    <t>Question</t>
-  </si>
-  <si>
-    <t>Answer</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -66,6 +104,12 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="1"/>
     </font>
@@ -90,10 +134,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -109,6 +155,12 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Артём Савосин" id="{9D63949E-4215-4691-AB7B-A0A30DCC34DB}" userId="15080e1520f1cce4" providerId="Windows Live"/>
+</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -406,84 +458,206 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="A2" dT="2026-03-09T09:51:21.66" personId="{9D63949E-4215-4691-AB7B-A0A30DCC34DB}" id="{1661D921-632C-430C-921D-9910BCE3059E}">
+    <text>писать вопрос здесь, а справа ответ на него
+(так можно писать вниз до бесконечности)</text>
+  </threadedComment>
+  <threadedComment ref="C2" dT="2026-03-09T09:50:01.38" personId="{9D63949E-4215-4691-AB7B-A0A30DCC34DB}" id="{955AFFB0-AFFE-458F-8DA4-B07AF093579C}">
+    <text>писать название здесь</text>
+  </threadedComment>
+  <threadedComment ref="D2" dT="2026-03-09T09:50:24.14" personId="{9D63949E-4215-4691-AB7B-A0A30DCC34DB}" id="{BFCD12D3-2FD0-414A-BD87-6586BD3166F9}">
+    <text xml:space="preserve">писать тему здесь
+</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:K40"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22">
-      <c r="A1" t="s">
+    <row r="1" spans="1:11">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
       <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
-        <v>2</v>
-      </c>
-      <c r="F1" t="s">
-        <v>3</v>
-      </c>
-      <c r="G1" t="s">
-        <v>2</v>
-      </c>
-      <c r="H1" t="s">
-        <v>3</v>
-      </c>
-      <c r="I1" t="s">
-        <v>2</v>
-      </c>
-      <c r="J1" t="s">
-        <v>3</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="P1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="R1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="T1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="V1" s="2" t="s">
-        <v>3</v>
-      </c>
+      <c r="K1" s="1"/>
+    </row>
+    <row r="2" spans="1:11">
+      <c r="A2" s="3"/>
+      <c r="B2" s="3"/>
+    </row>
+    <row r="3" spans="1:11">
+      <c r="A3" s="4"/>
+      <c r="B3" s="3"/>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="A4" s="3"/>
+      <c r="B4" s="3"/>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="A5" s="4"/>
+      <c r="B5" s="3"/>
+    </row>
+    <row r="6" spans="1:11">
+      <c r="A6" s="3"/>
+      <c r="B6" s="3"/>
+    </row>
+    <row r="7" spans="1:11">
+      <c r="A7" s="4"/>
+      <c r="B7" s="3"/>
+    </row>
+    <row r="8" spans="1:11">
+      <c r="A8" s="3"/>
+      <c r="B8" s="3"/>
+    </row>
+    <row r="9" spans="1:11">
+      <c r="A9" s="4"/>
+      <c r="B9" s="3"/>
+    </row>
+    <row r="10" spans="1:11">
+      <c r="A10" s="3"/>
+      <c r="B10" s="3"/>
+    </row>
+    <row r="11" spans="1:11">
+      <c r="A11" s="3"/>
+      <c r="B11" s="3"/>
+    </row>
+    <row r="12" spans="1:11">
+      <c r="A12" s="3"/>
+      <c r="B12" s="3"/>
+    </row>
+    <row r="13" spans="1:11">
+      <c r="A13" s="3"/>
+      <c r="B13" s="3"/>
+    </row>
+    <row r="14" spans="1:11">
+      <c r="A14" s="3"/>
+      <c r="B14" s="3"/>
+    </row>
+    <row r="15" spans="1:11">
+      <c r="A15" s="3"/>
+      <c r="B15" s="3"/>
+    </row>
+    <row r="16" spans="1:11">
+      <c r="A16" s="3"/>
+      <c r="B16" s="3"/>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" s="3"/>
+      <c r="B17" s="3"/>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" s="3"/>
+      <c r="B18" s="3"/>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" s="3"/>
+      <c r="B19" s="3"/>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20" s="3"/>
+      <c r="B20" s="3"/>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" s="3"/>
+      <c r="B21" s="3"/>
+    </row>
+    <row r="22" spans="1:2">
+      <c r="A22" s="3"/>
+      <c r="B22" s="3"/>
+    </row>
+    <row r="23" spans="1:2">
+      <c r="A23" s="3"/>
+      <c r="B23" s="3"/>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24" s="3"/>
+      <c r="B24" s="3"/>
+    </row>
+    <row r="25" spans="1:2">
+      <c r="A25" s="3"/>
+      <c r="B25" s="3"/>
+    </row>
+    <row r="26" spans="1:2">
+      <c r="A26" s="3"/>
+      <c r="B26" s="3"/>
+    </row>
+    <row r="27" spans="1:2">
+      <c r="A27" s="3"/>
+      <c r="B27" s="3"/>
+    </row>
+    <row r="28" spans="1:2">
+      <c r="A28" s="3"/>
+      <c r="B28" s="3"/>
+    </row>
+    <row r="29" spans="1:2">
+      <c r="A29" s="3"/>
+      <c r="B29" s="3"/>
+    </row>
+    <row r="30" spans="1:2">
+      <c r="A30" s="3"/>
+      <c r="B30" s="3"/>
+    </row>
+    <row r="31" spans="1:2">
+      <c r="A31" s="3"/>
+      <c r="B31" s="3"/>
+    </row>
+    <row r="32" spans="1:2">
+      <c r="A32" s="3"/>
+      <c r="B32" s="3"/>
+    </row>
+    <row r="33" spans="1:2">
+      <c r="A33" s="3"/>
+      <c r="B33" s="3"/>
+    </row>
+    <row r="34" spans="1:2">
+      <c r="A34" s="3"/>
+      <c r="B34" s="3"/>
+    </row>
+    <row r="35" spans="1:2">
+      <c r="A35" s="3"/>
+      <c r="B35" s="3"/>
+    </row>
+    <row r="36" spans="1:2">
+      <c r="A36" s="3"/>
+      <c r="B36" s="3"/>
+    </row>
+    <row r="37" spans="1:2">
+      <c r="A37" s="3"/>
+      <c r="B37" s="3"/>
+    </row>
+    <row r="38" spans="1:2">
+      <c r="A38" s="3"/>
+      <c r="B38" s="3"/>
+    </row>
+    <row r="39" spans="1:2">
+      <c r="A39" s="3"/>
+      <c r="B39" s="3"/>
+    </row>
+    <row r="40" spans="1:2">
+      <c r="A40" s="3"/>
+      <c r="B40" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>